<commit_message>
some changes in booking form as respect to parcel value , mainly change validationof parcel value
</commit_message>
<xml_diff>
--- a/public/file/Trax Book Omni Overall Shipment Template.xlsx
+++ b/public/file/Trax Book Omni Overall Shipment Template.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26227"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\sonic\public\file\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56EDBDAB-CC0B-4876-AB0B-3BD560142DFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3900" yWindow="3396" windowWidth="17280" windowHeight="8964"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="62">
   <si>
     <t>Consignee Name</t>
   </si>
@@ -207,12 +208,15 @@
   </si>
   <si>
     <t>Return Address Id</t>
+  </si>
+  <si>
+    <t>Parcel Value</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -558,8 +562,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:BI1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:BJ1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.44140625" style="1" bestFit="1" customWidth="1"/>
@@ -618,9 +622,10 @@
     <col min="55" max="59" width="24.5546875" bestFit="1" customWidth="1"/>
     <col min="60" max="60" width="14.33203125" customWidth="1"/>
     <col min="61" max="61" width="18.6640625" customWidth="1"/>
+    <col min="62" max="62" width="12.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:61" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:62" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
@@ -803,6 +808,9 @@
       </c>
       <c r="BI1" t="s">
         <v>60</v>
+      </c>
+      <c r="BJ1" t="s">
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>